<commit_message>
Laminas regeneradas (regeneracion completa del 2026-10-04), piramides 2018-2024, empates nombrados (#191) (graficos_dependencia)
</commit_message>
<xml_diff>
--- a/output/graficos_dependencia/plot_regional_d_deptot_a_2018_araucania.xlsx
+++ b/output/graficos_dependencia/plot_regional_d_deptot_a_2018_araucania.xlsx
@@ -38,7 +38,7 @@
     <t xml:space="preserve">Reg_Mujeres</t>
   </si>
   <si>
-    <t xml:space="preserve">Araucania</t>
+    <t xml:space="preserve">La Araucanía</t>
   </si>
   <si>
     <t xml:space="preserve">Campo</t>
@@ -50,7 +50,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-26 23:43</t>
+    <t xml:space="preserve">2026-10-05 04:52</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -74,7 +74,7 @@
     <t xml:space="preserve">Unidad territorial</t>
   </si>
   <si>
-    <t xml:space="preserve">Region de Araucania</t>
+    <t xml:space="preserve">Region de La Araucanía</t>
   </si>
   <si>
     <t xml:space="preserve">Año</t>
@@ -466,7 +466,7 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="12.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="14.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="10.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="10.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="11.71" hidden="0" customWidth="1"/>

</xml_diff>